<commit_message>
Add OAuth social login support: update .env.example for Google and GitHub credentials, enhance routing for OAuth callbacks in Routes.php, implement OAuth login handling in AuthService, and integrate OAuth login options in frontend components. Update login and registration pages to support OAuth authentication flow.
</commit_message>
<xml_diff>
--- a/writable/exports/analytics_report.xlsx
+++ b/writable/exports/analytics_report.xlsx
@@ -385,7 +385,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>31.85</v>
+        <v>47.07</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -393,7 +393,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>31.85</v>
+        <v>47.07</v>
       </c>
     </row>
     <row r="4" spans="1:2">

</xml_diff>